<commit_message>
Sprint 3 Mission completed data inspection module
</commit_message>
<xml_diff>
--- a/data/raw/数据表1.xlsx
+++ b/data/raw/数据表1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\qiang docment\Casino-AI-MVP\data\raw\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3DC5243E-D754-4911-B454-50DD20AA9B4B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6FBED7BB-40EC-4147-9DC6-20D028370E04}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="23236" windowHeight="13875" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="12">
   <si>
     <t>姓名</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -44,6 +44,34 @@
   </si>
   <si>
     <t>女</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>薪酬</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>胖子</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>男</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>爱德华</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>王尼玛</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>赵四</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>黄蓉</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -369,10 +397,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C2"/>
+  <dimension ref="A1:D7"/>
   <sheetFormatPr defaultRowHeight="13.9" x14ac:dyDescent="0.4"/>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -382,8 +410,11 @@
       <c r="C1" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="D1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -392,6 +423,79 @@
       </c>
       <c r="C2">
         <v>15</v>
+      </c>
+      <c r="D2">
+        <v>1500</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.4">
+      <c r="A3" t="s">
+        <v>6</v>
+      </c>
+      <c r="B3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C3">
+        <v>27</v>
+      </c>
+      <c r="D3">
+        <v>1876</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.4">
+      <c r="A4" t="s">
+        <v>8</v>
+      </c>
+      <c r="B4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C4">
+        <v>19</v>
+      </c>
+      <c r="D4">
+        <v>2400</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.4">
+      <c r="A5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B5" t="s">
+        <v>4</v>
+      </c>
+      <c r="C5">
+        <v>22</v>
+      </c>
+      <c r="D5">
+        <v>1980</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.4">
+      <c r="A6" t="s">
+        <v>10</v>
+      </c>
+      <c r="B6" t="s">
+        <v>7</v>
+      </c>
+      <c r="C6">
+        <v>24</v>
+      </c>
+      <c r="D6">
+        <v>2690</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.4">
+      <c r="A7" t="s">
+        <v>11</v>
+      </c>
+      <c r="B7" t="s">
+        <v>4</v>
+      </c>
+      <c r="C7">
+        <v>21</v>
+      </c>
+      <c r="D7">
+        <v>3890</v>
       </c>
     </row>
   </sheetData>

</xml_diff>